<commit_message>
fix(motor_matching): CONCEPTO column en Ambiguos para persistir correcciones sin MZ
Raíz del bug: _leer_validados_ambiguos descartaba entradas con MZ vacío
(if not mz: continue), por lo que correcciones CONCEPTO-only nunca llegaban
a trazabilidad Ambiguos y reaparecían como pendientes en el siguiente ciclo.

Cambios:
- exportar_motor.py: agrega columna CONCEPTO al sheet Ambiguos (colspan
  "¿CÓMO SE RESOLVIÓ?" sube de 2→3, alineado con Sin_identificar/Maestro_inexacto)
- main.py: actualiza _leer_validados_ambiguos, _leer_acum_ambiguos_traz y
  _leer_hoja_ambiguos para aceptar entradas con CONCEPTO pero sin MZ/LOTE
- docs/trazabilidad.html: documenta nueva columna CONCEPTO en sección Ambiguos
- trazabilidad_2026_06.xlsx: 4 filas en Ambiguos (Vilma x2 MZ+LOTE, Janet x2 CONCEPTO)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_pagos/yape/motor_matching/trazabilidad/trazabilidad_2026_06.xlsx
+++ b/4_pagos/yape/motor_matching/trazabilidad/trazabilidad_2026_06.xlsx
@@ -661,7 +661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -838,7 +838,7 @@
       </c>
       <c r="Q3" s="18" t="inlineStr">
         <is>
-          <t>15/06/2026 05:57</t>
+          <t>15/06/2026 06:14</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="Q4" s="18" t="inlineStr">
         <is>
-          <t>15/06/2026 05:57</t>
+          <t>15/06/2026 06:14</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="Q5" s="18" t="inlineStr">
         <is>
-          <t>15/06/2026 05:57</t>
+          <t>15/06/2026 06:14</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
       </c>
       <c r="Q6" s="18" t="inlineStr">
         <is>
-          <t>15/06/2026 05:57</t>
+          <t>15/06/2026 06:14</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="Q7" s="18" t="inlineStr">
         <is>
-          <t>15/06/2026 05:57</t>
+          <t>15/06/2026 06:14</t>
         </is>
       </c>
     </row>
@@ -1097,101 +1097,7 @@
       </c>
       <c r="Q8" s="18" t="inlineStr">
         <is>
-          <t>15/06/2026 05:57</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="11" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>TE PAGÓ</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>JANET VIL*</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr"/>
-      <c r="G9" s="13" t="n">
-        <v>152</v>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>geral cobro de agua</t>
-        </is>
-      </c>
-      <c r="I9" s="12" t="inlineStr">
-        <is>
-          <t>07/06/2026 10:39:56</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="15" t="inlineStr"/>
-      <c r="L9" s="15" t="inlineStr"/>
-      <c r="M9" s="16" t="inlineStr">
-        <is>
-          <t>cobro de agua (Yerald)</t>
-        </is>
-      </c>
-      <c r="N9" s="16" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr"/>
-      <c r="P9" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q9" s="18" t="inlineStr">
-        <is>
-          <t>15/06/2026 05:57</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="11" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>TE PAGÓ</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>JANET VIL*</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="inlineStr"/>
-      <c r="G10" s="13" t="n">
-        <v>450</v>
-      </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>350#1cobro 100 # cobro maximo</t>
-        </is>
-      </c>
-      <c r="I10" s="12" t="inlineStr">
-        <is>
-          <t>07/06/2026 10:39:01</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="15" t="inlineStr"/>
-      <c r="L10" s="15" t="inlineStr"/>
-      <c r="M10" s="16" t="inlineStr">
-        <is>
-          <t>cobro de agua (Maximo)</t>
-        </is>
-      </c>
-      <c r="N10" s="16" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
-      <c r="P10" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q10" s="18" t="inlineStr">
-        <is>
-          <t>15/06/2026 05:57</t>
+          <t>15/06/2026 06:14</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1227,9 +1133,10 @@
     <col width="1" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="1" customWidth="1" min="13" max="13"/>
-    <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="1" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1253,11 +1160,11 @@
       <c r="J1" s="2" t="inlineStr"/>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>ELEGIDO</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr"/>
-      <c r="N1" s="5" t="inlineStr">
+          <t>¿CÓMO SE RESOLVIÓ?</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr"/>
+      <c r="O1" s="5" t="inlineStr">
         <is>
           <t>¿CUÁNDO?</t>
         </is>
@@ -1312,13 +1219,18 @@
           <t>LOTE_FINAL</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>CONCEPTO</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>CICLO</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>FECHA_CORRECCION</t>
         </is>
@@ -1371,13 +1283,14 @@
           <t>3</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="17" t="n">
+      <c r="M3" s="16" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="O3" s="18" t="inlineStr">
-        <is>
-          <t>15/06/2026 05:57</t>
+      <c r="P3" s="18" t="inlineStr">
+        <is>
+          <t>15/06/2026 06:14</t>
         </is>
       </c>
     </row>
@@ -1428,22 +1341,131 @@
           <t>5</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="17" t="n">
+      <c r="M4" s="16" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="O4" s="18" t="inlineStr">
-        <is>
-          <t>15/06/2026 05:57</t>
+      <c r="P4" s="18" t="inlineStr">
+        <is>
+          <t>15/06/2026 06:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>U0118</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>RAQUEL MABEL AVILA MORALES</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Janet Vil*</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>152</v>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>geral cobro de agua</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>07/06/2026 10:39:56</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="21" t="inlineStr">
+        <is>
+          <t>G-3(123,+29) · W-19(89,+63) · T-10(79,+73) · G-21A(40,+112) · V-2(16,+136)</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="15" t="inlineStr"/>
+      <c r="L5" s="15" t="inlineStr"/>
+      <c r="M5" s="16" t="inlineStr">
+        <is>
+          <t>cobro de agua (Yerald)</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="P5" s="18" t="inlineStr">
+        <is>
+          <t>15/06/2026 06:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>U0118</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>RAQUEL MABEL AVILA MORALES</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Janet Vil*</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>450</v>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>350#1cobro 100 # cobro maximo</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>07/06/2026 10:39:01</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="21" t="inlineStr">
+        <is>
+          <t>G-3(123,+327) · W-19(89,+361) · T-10(79,+371) · G-21A(40,+410) · V-2(16,+434)</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="15" t="inlineStr"/>
+      <c r="L6" s="15" t="inlineStr"/>
+      <c r="M6" s="16" t="inlineStr">
+        <is>
+          <t>cobro de agua (Maximo)</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" s="18" t="inlineStr">
+        <is>
+          <t>15/06/2026 06:14</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="O1:P1"/>
     <mergeCell ref="D1:G1"/>
-    <mergeCell ref="K1:L1"/>
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="K1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1774,7 +1796,7 @@
       </c>
       <c r="R3" s="18" t="inlineStr">
         <is>
-          <t>15/06/2026 05:57</t>
+          <t>15/06/2026 06:14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(motor_matching): Pagos_comunitarios — desglose de pagos de directivos por lote
Detecta pagos comunitarios (un directivo cobra varios lotes) vía
CONCEPTO=comunitario en Ambiguos. Nueva hoja Pagos_comunitarios en
pendientes y trazabilidad: el operador parte el monto por lote y el
motor emite una fila tepago por lote. Incluye MENSAJE del banco como
referencia. Convención Title_Case para hojas Excel en CLAUDE.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_pagos/yape/motor_matching/trazabilidad/trazabilidad_2026_06.xlsx
+++ b/4_pagos/yape/motor_matching/trazabilidad/trazabilidad_2026_06.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambiguos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pagos_multiples" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maestro_inexacto" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pagos_comunitarios" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -114,8 +115,19 @@
       <color rgb="00A32D2D"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009A3412"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00065F46"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -170,6 +182,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFBF0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF7ED"/>
       </patternFill>
     </fill>
   </fills>
@@ -227,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -295,6 +312,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -661,7 +690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -838,7 +867,7 @@
       </c>
       <c r="Q3" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
@@ -893,7 +922,7 @@
       </c>
       <c r="Q4" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
@@ -944,7 +973,7 @@
       </c>
       <c r="Q5" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
@@ -987,7 +1016,7 @@
       </c>
       <c r="Q6" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1071,7 @@
       </c>
       <c r="Q7" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1126,7 @@
       </c>
       <c r="Q8" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1181,117 @@
       </c>
       <c r="Q9" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>U0065</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>ANALY QUINECHE MORANTE</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>TE PAGÓ</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>PLIN - ANALI QUINECHE</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr"/>
+      <c r="G10" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="H10" s="14" t="inlineStr"/>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>18/06/2026 21:01:29</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L10" s="15" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="M10" s="16" t="inlineStr"/>
+      <c r="N10" s="16" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q10" s="18" t="inlineStr">
+        <is>
+          <t>29/06/2026 09:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>U0102</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>MARIA GODO SIFUENTES</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>TE PAGÓ</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>PLIN - ELIAS AGAPITO SALES BLAS</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr"/>
+      <c r="G11" s="13" t="n">
+        <v>41</v>
+      </c>
+      <c r="H11" s="14" t="inlineStr"/>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>17/06/2026 20:32:08</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L11" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M11" s="16" t="inlineStr"/>
+      <c r="N11" s="16" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q11" s="18" t="inlineStr">
+        <is>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1484,7 @@
       </c>
       <c r="P3" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
@@ -1403,73 +1542,77 @@
       </c>
       <c r="P4" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>U0118</t>
+          <t>U0092</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>RAQUEL MABEL AVILA MORALES</t>
+          <t>GREGORIO TRUJILLO LEON</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Janet Vil*</t>
+          <t>Wilder Tru*</t>
         </is>
       </c>
       <c r="E5" s="13" t="n">
-        <v>152</v>
+        <v>44</v>
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>geral cobro de agua</t>
+          <t>Vicky Masías. W4?</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>07/06/2026 10:39:56</t>
+          <t>15/06/2026 21:13:40</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="21" t="inlineStr">
         <is>
-          <t>G-3(123,+29) · W-19(89,+63) · T-10(79,+73) · G-21A(40,+112) · V-2(16,+136)</t>
+          <t>E-7(0.0,+9999) · M-18(0.0,+9999) · P-11A(0.0,+9999)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="15" t="inlineStr"/>
-      <c r="L5" s="15" t="inlineStr"/>
-      <c r="M5" s="16" t="inlineStr">
-        <is>
-          <t>cobro de agua (Yerald)</t>
-        </is>
-      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="M5" s="16" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="17" t="n">
         <v>2</v>
       </c>
       <c r="P5" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>U0118</t>
+          <t>U0137</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>RAQUEL MABEL AVILA MORALES</t>
+          <t>DEYSI COSME GARCILAZO</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -1479,22 +1622,22 @@
         </is>
       </c>
       <c r="E6" s="13" t="n">
-        <v>450</v>
+        <v>152</v>
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>350#1cobro 100 # cobro maximo</t>
+          <t>geral cobro de agua</t>
         </is>
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>07/06/2026 10:39:01</t>
+          <t>07/06/2026 10:39:56</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="21" t="inlineStr">
         <is>
-          <t>G-3(123,+327) · W-19(89,+361) · T-10(79,+371) · G-21A(40,+410) · V-2(16,+434)</t>
+          <t>G-21A(0.0,+9999) · G-3(0.0,+9999) · T-10(0.0,+9999) · V-2(0.0,+9999) · W-19(0.0,+9999)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
@@ -1502,7 +1645,7 @@
       <c r="L6" s="15" t="inlineStr"/>
       <c r="M6" s="16" t="inlineStr">
         <is>
-          <t>cobro de agua (Maximo)</t>
+          <t>comunitario</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr"/>
@@ -1511,65 +1654,61 @@
       </c>
       <c r="P6" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>U0092</t>
+          <t>U0137</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>GREGORIO TRUJILLO LEON</t>
+          <t>DEYSI COSME GARCILAZO</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Wilder Tru*</t>
+          <t>Janet Vil*</t>
         </is>
       </c>
       <c r="E7" s="13" t="n">
-        <v>44</v>
+        <v>450</v>
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Vicky Masías. W4?</t>
+          <t>350#1cobro 100 # cobro maximo</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>15/06/2026 21:13:40</t>
+          <t>07/06/2026 10:39:01</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="21" t="inlineStr">
         <is>
-          <t>E-7(0.0,+9999) · M-18(0.0,+9999) · P-11A(0.0,+9999)</t>
+          <t>G-21A(0.0,+9999) · G-3(0.0,+9999) · T-10(0.0,+9999) · V-2(0.0,+9999) · W-19(0.0,+9999)</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="15" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="L7" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="M7" s="16" t="inlineStr"/>
+      <c r="K7" s="15" t="inlineStr"/>
+      <c r="L7" s="15" t="inlineStr"/>
+      <c r="M7" s="16" t="inlineStr">
+        <is>
+          <t>comunitario</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="17" t="n">
         <v>2</v>
       </c>
       <c r="P7" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
@@ -1909,7 +2048,7 @@
       </c>
       <c r="R3" s="18" t="inlineStr">
         <is>
-          <t>17/06/2026 20:27</t>
+          <t>29/06/2026 09:04</t>
         </is>
       </c>
     </row>
@@ -1922,4 +2061,459 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="1" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="1" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="1" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>¿QUIÉN ES?</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr"/>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>¿QUÉ HIZO EL BANCO?</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr"/>
+      <c r="H1" s="24" t="inlineStr">
+        <is>
+          <t>DESGLOSE COMUNITARIO</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr"/>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>¿CUÁNDO?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>USER_ID</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>NOMBRE</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>ORIGEN</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>FECHA</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>MONTO_TOTAL</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="22" t="inlineStr">
+        <is>
+          <t>MZ</t>
+        </is>
+      </c>
+      <c r="I2" s="22" t="inlineStr">
+        <is>
+          <t>LOTE</t>
+        </is>
+      </c>
+      <c r="J2" s="22" t="inlineStr">
+        <is>
+          <t>MONTO_PARCIAL</t>
+        </is>
+      </c>
+      <c r="K2" s="22" t="inlineStr">
+        <is>
+          <t>MOTIVO</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>CICLO</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>FECHA_CORRECCION</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>U0199</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>NIEVES CUZCO VALLE DE LEON</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Janet Vil*</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>07/06/2026 10:39:56</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>152</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="25" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="I3" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="J3" s="26" t="n">
+        <v>30</v>
+      </c>
+      <c r="K3" s="27" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N3" s="18" t="inlineStr">
+        <is>
+          <t>29/06/2026 09:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>U0472</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>ANI CRUZ DOMINGUEZ</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Janet Vil*</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>07/06/2026 10:39:56</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>152</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="25" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="I4" s="25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J4" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="K4" s="27" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" s="18" t="inlineStr">
+        <is>
+          <t>29/06/2026 09:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="10" t="inlineStr"/>
+      <c r="B5" s="11" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Janet Vil*</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>07/06/2026 10:39:56</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>152</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="25" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="I5" s="25" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="J5" s="26" t="n">
+        <v>89</v>
+      </c>
+      <c r="K5" s="27" t="inlineStr">
+        <is>
+          <t>devolucion_cobradora_yeral se confundio yapeo de mas</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N5" s="18" t="inlineStr">
+        <is>
+          <t>29/06/2026 09:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>U0480</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>ESTELA FLORES LOAYZA</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Janet Vil*</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>07/06/2026 10:39:56</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>152</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="25" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="I6" s="25" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="J6" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="K6" s="27" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="18" t="inlineStr">
+        <is>
+          <t>29/06/2026 09:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="10" t="inlineStr"/>
+      <c r="B7" s="11" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Janet Vil*</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>07/06/2026 10:39:01</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>450</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="25" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="I7" s="25" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="J7" s="26" t="n">
+        <v>200</v>
+      </c>
+      <c r="K7" s="27" t="inlineStr">
+        <is>
+          <t>ira a una hoja seguimiento de tanque en el futuro</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" s="18" t="inlineStr">
+        <is>
+          <t>29/06/2026 09:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="10" t="inlineStr"/>
+      <c r="B8" s="11" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Janet Vil*</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>07/06/2026 10:39:01</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="n">
+        <v>450</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="25" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="I8" s="25" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="J8" s="26" t="n">
+        <v>200</v>
+      </c>
+      <c r="K8" s="27" t="inlineStr">
+        <is>
+          <t>ira a una hoja seguimiento de tanque en el futuro</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" s="18" t="inlineStr">
+        <is>
+          <t>29/06/2026 09:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="10" t="inlineStr"/>
+      <c r="B9" s="11" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Janet Vil*</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>07/06/2026 10:39:01</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>450</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="25" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="I9" s="25" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="J9" s="26" t="n">
+        <v>50</v>
+      </c>
+      <c r="K9" s="27" t="inlineStr">
+        <is>
+          <t>ira a una hoja seguimiento de tanque en el futuro</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" s="18" t="inlineStr">
+        <is>
+          <t>29/06/2026 09:04</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="H1:K1"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: seguimiento_pueblo (event-sourced) + arrastre_consolidado + módulo 7_cierre
seguimiento_pueblo reemplaza el saldo estático de MULTA/ACUERDOS/CONVENIO por un
ledger append-only (CARGO/PAGO/AJUSTE), sembrado desde DATA_boletas +
medidor_saldo + inscripcion_saldo. 2_planilla (Opción A, writer único) lee el
consolidado de 5_cobranza en vivo para agua+corte y el ledger para los 3
conceptos de seguimiento.

7_cierre (nuevo): transiciona un período cerrado — GATE (ciclo validado) →
COSECHAR (foto inmutable a archivo/YYYY-MM/) → FREEZE (estado_ciclo=CERRADO) →
LIMPIAR (reset de mesa_*/correcciones_lote a template). Doble seguro: dry-run
por defecto, --confirmar + consentimiento tipeado para la parte irreversible.

Extraídos a shared/ (cross-módulo, 3+ llamadores): utils_estado_ciclo.py
(gate/freeze de estado_ciclo.json, antes duplicado en 3 módulos),
utils_templates.py (template de mesa_N), utils_lote.py +escribir vacío.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_pagos/yape/motor_matching/trazabilidad/trazabilidad_2026_06.xlsx
+++ b/4_pagos/yape/motor_matching/trazabilidad/trazabilidad_2026_06.xlsx
@@ -244,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -323,6 +323,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -867,7 +870,7 @@
       </c>
       <c r="Q3" s="18" t="inlineStr">
         <is>
-          <t>29/06/2026 09:04</t>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -922,7 +925,7 @@
       </c>
       <c r="Q4" s="18" t="inlineStr">
         <is>
-          <t>29/06/2026 09:04</t>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -973,7 +976,7 @@
       </c>
       <c r="Q5" s="18" t="inlineStr">
         <is>
-          <t>29/06/2026 09:04</t>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1019,7 @@
       </c>
       <c r="Q6" s="18" t="inlineStr">
         <is>
-          <t>29/06/2026 09:04</t>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1074,7 @@
       </c>
       <c r="Q7" s="18" t="inlineStr">
         <is>
-          <t>29/06/2026 09:04</t>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1129,7 @@
       </c>
       <c r="Q8" s="18" t="inlineStr">
         <is>
-          <t>29/06/2026 09:04</t>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1184,7 @@
       </c>
       <c r="Q9" s="18" t="inlineStr">
         <is>
-          <t>29/06/2026 09:04</t>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1239,7 @@
       </c>
       <c r="Q10" s="18" t="inlineStr">
         <is>
-          <t>29/06/2026 09:04</t>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1294,7 @@
       </c>
       <c r="Q11" s="18" t="inlineStr">
         <is>
-          <t>29/06/2026 09:04</t>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1328,9 +1331,10 @@
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="1" customWidth="1" min="14" max="14"/>
-    <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="1" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1357,8 +1361,8 @@
           <t>¿CÓMO SE RESOLVIÓ?</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr"/>
-      <c r="O1" s="5" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr"/>
+      <c r="P1" s="5" t="inlineStr">
         <is>
           <t>¿CUÁNDO?</t>
         </is>
@@ -1418,13 +1422,18 @@
           <t>CONCEPTO</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="N2" s="9" t="inlineStr">
+        <is>
+          <t>ESTADO_REGISTRO</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>CICLO</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="Q2" s="5" t="inlineStr">
         <is>
           <t>FECHA_CORRECCION</t>
         </is>
@@ -1478,13 +1487,18 @@
         </is>
       </c>
       <c r="M3" s="16" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="17" t="n">
+      <c r="N3" s="15" t="inlineStr">
+        <is>
+          <t>REGISTRO_NORMAL</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="P3" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q3" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1536,13 +1550,18 @@
         </is>
       </c>
       <c r="M4" s="16" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="17" t="n">
+      <c r="N4" s="15" t="inlineStr">
+        <is>
+          <t>REGISTRO_NORMAL</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="P4" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q4" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1594,13 +1613,18 @@
         </is>
       </c>
       <c r="M5" s="16" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
-      <c r="O5" s="17" t="n">
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>REGISTRO_NORMAL</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="P5" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q5" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1648,13 +1672,18 @@
           <t>comunitario</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="17" t="n">
+      <c r="N6" s="15" t="inlineStr">
+        <is>
+          <t>PADRE_SEGREGADO</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="P6" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q6" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1702,22 +1731,27 @@
           <t>comunitario</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="17" t="n">
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>PADRE_SEGREGADO</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="P7" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q7" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="P1:Q1"/>
     <mergeCell ref="D1:G1"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="K1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2048,7 +2082,7 @@
       </c>
       <c r="R3" s="18" t="inlineStr">
         <is>
-          <t>29/06/2026 09:04</t>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2069,7 +2103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2083,9 +2117,12 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="1" customWidth="1" min="12" max="12"/>
-    <col width="7" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="1" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -2106,8 +2143,8 @@
           <t>DESGLOSE COMUNITARIO</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr"/>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr"/>
+      <c r="P1" s="5" t="inlineStr">
         <is>
           <t>¿CUÁNDO?</t>
         </is>
@@ -2161,13 +2198,28 @@
           <t>MOTIVO</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="L2" s="22" t="inlineStr">
+        <is>
+          <t>CONCEPTO</t>
+        </is>
+      </c>
+      <c r="M2" s="22" t="inlineStr">
+        <is>
+          <t>ESTADO_REGISTRO</t>
+        </is>
+      </c>
+      <c r="N2" s="22" t="inlineStr">
+        <is>
+          <t>ID_PADRE</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>CICLO</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="Q2" s="5" t="inlineStr">
         <is>
           <t>FECHA_CORRECCION</t>
         </is>
@@ -2213,13 +2265,24 @@
         <v>30</v>
       </c>
       <c r="K3" s="27" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="17" t="n">
+      <c r="L3" s="27" t="inlineStr"/>
+      <c r="M3" s="25" t="inlineStr">
+        <is>
+          <t>HIJO_SEGREGADO</t>
+        </is>
+      </c>
+      <c r="N3" s="28" t="inlineStr">
+        <is>
+          <t>JANET VIL*|07/06/2026 10:39:56</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="N3" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q3" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2263,13 +2326,24 @@
         <v>25</v>
       </c>
       <c r="K4" s="27" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="17" t="n">
+      <c r="L4" s="27" t="inlineStr"/>
+      <c r="M4" s="25" t="inlineStr">
+        <is>
+          <t>HIJO_SEGREGADO</t>
+        </is>
+      </c>
+      <c r="N4" s="28" t="inlineStr">
+        <is>
+          <t>JANET VIL*|07/06/2026 10:39:56</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="N4" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q4" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2304,18 +2378,25 @@
       <c r="J5" s="26" t="n">
         <v>89</v>
       </c>
-      <c r="K5" s="27" t="inlineStr">
-        <is>
-          <t>devolucion_cobradora_yeral se confundio yapeo de mas</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="17" t="n">
+      <c r="K5" s="27" t="inlineStr"/>
+      <c r="L5" s="27" t="inlineStr"/>
+      <c r="M5" s="25" t="inlineStr">
+        <is>
+          <t>HIJO_SEGREGADO</t>
+        </is>
+      </c>
+      <c r="N5" s="28" t="inlineStr">
+        <is>
+          <t>JANET VIL*|07/06/2026 10:39:56</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="N5" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q5" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2359,19 +2440,38 @@
         <v>8</v>
       </c>
       <c r="K6" s="27" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="17" t="n">
+      <c r="L6" s="27" t="inlineStr"/>
+      <c r="M6" s="25" t="inlineStr">
+        <is>
+          <t>HIJO_SEGREGADO</t>
+        </is>
+      </c>
+      <c r="N6" s="28" t="inlineStr">
+        <is>
+          <t>JANET VIL*|07/06/2026 10:39:56</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="N6" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q6" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="11" t="inlineStr"/>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>U0271</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>MARIA HUERTA MILLA</t>
+        </is>
+      </c>
       <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="12" t="inlineStr">
         <is>
@@ -2389,35 +2489,54 @@
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="25" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>O</t>
         </is>
       </c>
       <c r="I7" s="25" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J7" s="26" t="n">
         <v>200</v>
       </c>
-      <c r="K7" s="27" t="inlineStr">
-        <is>
-          <t>ira a una hoja seguimiento de tanque en el futuro</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="17" t="n">
+      <c r="K7" s="27" t="inlineStr"/>
+      <c r="L7" s="27" t="inlineStr">
+        <is>
+          <t>tanque</t>
+        </is>
+      </c>
+      <c r="M7" s="25" t="inlineStr">
+        <is>
+          <t>HIJO_SEGREGADO</t>
+        </is>
+      </c>
+      <c r="N7" s="28" t="inlineStr">
+        <is>
+          <t>JANET VIL*|07/06/2026 10:39:01</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="N7" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q7" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="11" t="inlineStr"/>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>U0272</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>REYNA HUERTA MILLA</t>
+        </is>
+      </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="12" t="inlineStr">
         <is>
@@ -2435,29 +2554,40 @@
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="25" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>O</t>
         </is>
       </c>
       <c r="I8" s="25" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J8" s="26" t="n">
         <v>200</v>
       </c>
-      <c r="K8" s="27" t="inlineStr">
-        <is>
-          <t>ira a una hoja seguimiento de tanque en el futuro</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="17" t="n">
+      <c r="K8" s="27" t="inlineStr"/>
+      <c r="L8" s="27" t="inlineStr">
+        <is>
+          <t>tanque</t>
+        </is>
+      </c>
+      <c r="M8" s="25" t="inlineStr">
+        <is>
+          <t>HIJO_SEGREGADO</t>
+        </is>
+      </c>
+      <c r="N8" s="28" t="inlineStr">
+        <is>
+          <t>JANET VIL*|07/06/2026 10:39:01</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="N8" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q8" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2492,26 +2622,37 @@
       <c r="J9" s="26" t="n">
         <v>50</v>
       </c>
-      <c r="K9" s="27" t="inlineStr">
-        <is>
-          <t>ira a una hoja seguimiento de tanque en el futuro</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="17" t="n">
+      <c r="K9" s="27" t="inlineStr"/>
+      <c r="L9" s="27" t="inlineStr">
+        <is>
+          <t>tanque</t>
+        </is>
+      </c>
+      <c r="M9" s="25" t="inlineStr">
+        <is>
+          <t>HIJO_SEGREGADO</t>
+        </is>
+      </c>
+      <c r="N9" s="28" t="inlineStr">
+        <is>
+          <t>JANET VIL*|07/06/2026 10:39:01</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr"/>
+      <c r="P9" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="N9" s="18" t="inlineStr">
-        <is>
-          <t>29/06/2026 09:04</t>
+      <c r="Q9" s="18" t="inlineStr">
+        <is>
+          <t>30/06/2026 16:24</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="H1:K1"/>
+    <mergeCell ref="P1:Q1"/>
     <mergeCell ref="D1:F1"/>
+    <mergeCell ref="H1:N1"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>